<commit_message>
Fix micro element calculations
- Micro QTY is in grams (factor *1), not kg (*1000)
- Mn/Zn/B/Cu/Mo use Tank B capacity
- Fe-chelates use Tank A capacity
- Dose based on Tank B dilution (1000/B_dilution)

Matches original Excel spreadsheet formulas exactly.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FertiCalc_data.xlsx
+++ b/FertiCalc_data.xlsx
@@ -1759,12 +1759,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>test</t>
+          <t>test2</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>test</t>
+          <t>test2</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1774,7 +1774,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-23 10:26</t>
+          <t>2026-03-23 10:52</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -1813,7 +1813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1852,11 +1852,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>potassium-chloride</t>
+          <t>calcium-chloride</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -1865,11 +1865,76 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>potassium-chloride</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>potassium-nitrate-a</t>
         </is>
       </c>
-      <c r="C4" t="n">
-        <v>444</v>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>magnesium-nitrate-a</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>magnesium-nitrate-liquid-a</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ammonium-nitrate-a</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>nitric-acid-a</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>